<commit_message>
chore(quan-ly): cập nhật tiến độ dự án ngày 26/10
</commit_message>
<xml_diff>
--- a/quan-ly-du-an/quan-ly-du-an.xlsx
+++ b/quan-ly-du-an/quan-ly-du-an.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Esclipe_Web\Quan ly du an HTTT\quan-ly-du-an\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D70FAC-BDC1-4185-821A-3B8793BE59D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3655C91-85D1-47BB-B424-8247AAD608DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1848" yWindow="1848" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -627,7 +627,7 @@
     <t>Tối thiểu 20 trang ruột</t>
   </si>
   <si>
-    <t>Chưa kiểm tra</t>
+    <t>Đạt (ước tính 35–40 trang)</t>
   </si>
   <si>
     <t>Chữ trong bảng, hình là tiếng Việt</t>
@@ -675,7 +675,7 @@
     <t>Ghi chú đọc bài báo, thuật ngữ, điểm mâu thuẫn, tài liệu tham khảo</t>
   </si>
   <si>
-    <t>Nhập số liệu, script kiểm tra số liệu, khung LaTeX, Chương 1–2, sơ đồ</t>
+    <t>Số liệu, kiểm tra số liệu, mô phỏng, PLS-SEM, Monte Carlo, Excel/MS Project, Chương 1–4</t>
   </si>
   <si>
     <t>Tổng</t>
@@ -1652,7 +1652,7 @@
       <c r="H13" s="6"/>
       <c r="I13" s="9">
         <f>IFERROR(SUMPRODUCT(I14:I18,J14:J18)/SUM(J14:J18),0)</f>
-        <v>0.33333333333333331</v>
+        <v>1</v>
       </c>
       <c r="J13" s="8">
         <f>SUM(J14:J18)</f>
@@ -1763,25 +1763,29 @@
       <c r="D16" s="12">
         <v>46322</v>
       </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
+      <c r="E16" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F16" s="12">
+        <v>46321</v>
+      </c>
       <c r="G16" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H16" s="14" t="str">
+      <c r="H16" s="14">
         <f>IF(F16="","",F16-D16)</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="I16" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="16">
         <v>4</v>
       </c>
       <c r="K16" s="10" t="str">
         <f>IF(I16&gt;=1,"Hoàn thành",IF(I16&gt;0,"Đang làm",IF(D16&lt;$B$2,"Trễ hạn","Chưa bắt đầu")))</f>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L16" s="11" t="s">
         <v>49</v>
@@ -1803,25 +1807,29 @@
       <c r="D17" s="12">
         <v>46322</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
+      <c r="E17" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F17" s="12">
+        <v>46321</v>
+      </c>
       <c r="G17" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="14" t="str">
+      <c r="H17" s="14">
         <f>IF(F17="","",F17-D17)</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="I17" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="16">
         <v>4</v>
       </c>
       <c r="K17" s="10" t="str">
         <f>IF(I17&gt;=1,"Hoàn thành",IF(I17&gt;0,"Đang làm",IF(D17&lt;$B$2,"Trễ hạn","Chưa bắt đầu")))</f>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L17" s="11" t="s">
         <v>52</v>
@@ -1843,25 +1851,29 @@
       <c r="D18" s="12">
         <v>46323</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
+      <c r="E18" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F18" s="12">
+        <v>46321</v>
+      </c>
       <c r="G18" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H18" s="14" t="str">
+      <c r="H18" s="14">
         <f>IF(F18="","",F18-D18)</f>
-        <v/>
+        <v>-2</v>
       </c>
       <c r="I18" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" s="16">
         <v>8</v>
       </c>
       <c r="K18" s="10" t="str">
         <f>IF(I18&gt;=1,"Hoàn thành",IF(I18&gt;0,"Đang làm",IF(D18&lt;$B$2,"Trễ hạn","Chưa bắt đầu")))</f>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L18" s="11" t="s">
         <v>55</v>
@@ -1894,7 +1906,7 @@
       <c r="H19" s="6"/>
       <c r="I19" s="9">
         <f>IFERROR(SUMPRODUCT(I20:I28,J20:J28)/SUM(J20:J28),0)</f>
-        <v>0.34615384615384615</v>
+        <v>0.9538461538461539</v>
       </c>
       <c r="J19" s="8">
         <f>SUM(J20:J28)</f>
@@ -2093,25 +2105,29 @@
       <c r="D24" s="12">
         <v>46324</v>
       </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
+      <c r="E24" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F24" s="12">
+        <v>46321</v>
+      </c>
       <c r="G24" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H24" s="14" t="str">
+      <c r="H24" s="14">
         <f t="shared" si="1"/>
-        <v/>
+        <v>-3</v>
       </c>
       <c r="I24" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="16">
         <v>8</v>
       </c>
       <c r="K24" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L24" s="11" t="s">
         <v>73</v>
@@ -2133,25 +2149,29 @@
       <c r="D25" s="12">
         <v>46325</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
+      <c r="E25" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F25" s="12">
+        <v>46321</v>
+      </c>
       <c r="G25" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="14" t="str">
+      <c r="H25" s="14">
         <f t="shared" si="1"/>
-        <v/>
+        <v>-4</v>
       </c>
       <c r="I25" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" s="16">
         <v>6</v>
       </c>
       <c r="K25" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L25" s="11" t="s">
         <v>76</v>
@@ -2173,25 +2193,29 @@
       <c r="D26" s="12">
         <v>46326</v>
       </c>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
+      <c r="E26" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F26" s="12">
+        <v>46321</v>
+      </c>
       <c r="G26" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H26" s="14" t="str">
+      <c r="H26" s="14">
         <f t="shared" si="1"/>
-        <v/>
+        <v>-5</v>
       </c>
       <c r="I26" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" s="16">
         <v>8</v>
       </c>
       <c r="K26" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L26" s="11" t="s">
         <v>76</v>
@@ -2213,25 +2237,29 @@
       <c r="D27" s="12">
         <v>46327</v>
       </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
+      <c r="E27" s="12">
+        <v>46321</v>
+      </c>
+      <c r="F27" s="12">
+        <v>46321</v>
+      </c>
       <c r="G27" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="14" t="str">
+      <c r="H27" s="14">
         <f t="shared" si="1"/>
-        <v/>
+        <v>-6</v>
       </c>
       <c r="I27" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" s="16">
         <v>6</v>
       </c>
       <c r="K27" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Chưa bắt đầu</v>
+        <v>Hoàn thành</v>
       </c>
       <c r="L27" s="11" t="s">
         <v>76</v>
@@ -2253,7 +2281,9 @@
       <c r="D28" s="12">
         <v>46328</v>
       </c>
-      <c r="E28" s="12"/>
+      <c r="E28" s="12">
+        <v>46321</v>
+      </c>
       <c r="F28" s="12"/>
       <c r="G28" s="13">
         <f t="shared" si="0"/>
@@ -2264,14 +2294,14 @@
         <v/>
       </c>
       <c r="I28" s="15">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J28" s="16">
         <v>6</v>
       </c>
       <c r="K28" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Chưa bắt đầu</v>
+        <v>Đang làm</v>
       </c>
       <c r="L28" s="11" t="s">
         <v>83</v>
@@ -2516,7 +2546,7 @@
       </c>
       <c r="I36" s="18">
         <f>(I6*J6+I9*J9+I13*J13+I19*J19+I29*J29+I33*J33)/(J6+J9+J13+J19+J29+J33)</f>
-        <v>0.42574257425742573</v>
+        <v>0.89702970297029694</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
@@ -3515,7 +3545,7 @@
       </c>
       <c r="K15" s="22" t="str">
         <f>IF(WBS!$C16="","",IF(AND(WBS!$E16&lt;&gt;"",K$4&gt;=WBS!$E16,K$4&lt;=WBS!$F16),"■",IF(AND(K$4&gt;=WBS!$C16,K$4&lt;=WBS!$D16),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L15" s="22" t="str">
         <f>IF(WBS!$C16="","",IF(AND(WBS!$E16&lt;&gt;"",L$4&gt;=WBS!$E16,L$4&lt;=WBS!$F16),"■",IF(AND(L$4&gt;=WBS!$C16,L$4&lt;=WBS!$D16),"□","")))</f>
@@ -3597,7 +3627,7 @@
       </c>
       <c r="K16" s="22" t="str">
         <f>IF(WBS!$C17="","",IF(AND(WBS!$E17&lt;&gt;"",K$4&gt;=WBS!$E17,K$4&lt;=WBS!$F17),"■",IF(AND(K$4&gt;=WBS!$C17,K$4&lt;=WBS!$D17),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L16" s="22" t="str">
         <f>IF(WBS!$C17="","",IF(AND(WBS!$E17&lt;&gt;"",L$4&gt;=WBS!$E17,L$4&lt;=WBS!$F17),"■",IF(AND(L$4&gt;=WBS!$C17,L$4&lt;=WBS!$D17),"□","")))</f>
@@ -3679,7 +3709,7 @@
       </c>
       <c r="K17" s="22" t="str">
         <f>IF(WBS!$C18="","",IF(AND(WBS!$E18&lt;&gt;"",K$4&gt;=WBS!$E18,K$4&lt;=WBS!$F18),"■",IF(AND(K$4&gt;=WBS!$C18,K$4&lt;=WBS!$D18),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L17" s="22" t="str">
         <f>IF(WBS!$C18="","",IF(AND(WBS!$E18&lt;&gt;"",L$4&gt;=WBS!$E18,L$4&lt;=WBS!$F18),"■",IF(AND(L$4&gt;=WBS!$C18,L$4&lt;=WBS!$D18),"□","")))</f>
@@ -4171,7 +4201,7 @@
       </c>
       <c r="K23" s="22" t="str">
         <f>IF(WBS!$C24="","",IF(AND(WBS!$E24&lt;&gt;"",K$4&gt;=WBS!$E24,K$4&lt;=WBS!$F24),"■",IF(AND(K$4&gt;=WBS!$C24,K$4&lt;=WBS!$D24),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L23" s="22" t="str">
         <f>IF(WBS!$C24="","",IF(AND(WBS!$E24&lt;&gt;"",L$4&gt;=WBS!$E24,L$4&lt;=WBS!$F24),"■",IF(AND(L$4&gt;=WBS!$C24,L$4&lt;=WBS!$D24),"□","")))</f>
@@ -4253,7 +4283,7 @@
       </c>
       <c r="K24" s="22" t="str">
         <f>IF(WBS!$C25="","",IF(AND(WBS!$E25&lt;&gt;"",K$4&gt;=WBS!$E25,K$4&lt;=WBS!$F25),"■",IF(AND(K$4&gt;=WBS!$C25,K$4&lt;=WBS!$D25),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L24" s="22" t="str">
         <f>IF(WBS!$C25="","",IF(AND(WBS!$E25&lt;&gt;"",L$4&gt;=WBS!$E25,L$4&lt;=WBS!$F25),"■",IF(AND(L$4&gt;=WBS!$C25,L$4&lt;=WBS!$D25),"□","")))</f>
@@ -4335,7 +4365,7 @@
       </c>
       <c r="K25" s="22" t="str">
         <f>IF(WBS!$C26="","",IF(AND(WBS!$E26&lt;&gt;"",K$4&gt;=WBS!$E26,K$4&lt;=WBS!$F26),"■",IF(AND(K$4&gt;=WBS!$C26,K$4&lt;=WBS!$D26),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L25" s="22" t="str">
         <f>IF(WBS!$C26="","",IF(AND(WBS!$E26&lt;&gt;"",L$4&gt;=WBS!$E26,L$4&lt;=WBS!$F26),"■",IF(AND(L$4&gt;=WBS!$C26,L$4&lt;=WBS!$D26),"□","")))</f>
@@ -4417,7 +4447,7 @@
       </c>
       <c r="K26" s="22" t="str">
         <f>IF(WBS!$C27="","",IF(AND(WBS!$E27&lt;&gt;"",K$4&gt;=WBS!$E27,K$4&lt;=WBS!$F27),"■",IF(AND(K$4&gt;=WBS!$C27,K$4&lt;=WBS!$D27),"□","")))</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L26" s="22" t="str">
         <f>IF(WBS!$C27="","",IF(AND(WBS!$E27&lt;&gt;"",L$4&gt;=WBS!$E27,L$4&lt;=WBS!$F27),"■",IF(AND(L$4&gt;=WBS!$C27,L$4&lt;=WBS!$D27),"□","")))</f>
@@ -5559,11 +5589,11 @@
         <v>2.5</v>
       </c>
       <c r="C5" s="15">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D5" s="27">
         <f>B5*C5</f>
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>175</v>
@@ -5577,11 +5607,11 @@
         <v>2.5</v>
       </c>
       <c r="C6" s="15">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="D6" s="27">
         <f>B6*C6</f>
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>177</v>
@@ -5595,11 +5625,11 @@
         <v>2</v>
       </c>
       <c r="C7" s="15">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="27">
         <f>B7*C7</f>
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>179</v>
@@ -5651,11 +5681,11 @@
       </c>
       <c r="C10" s="28">
         <f>D10/B10</f>
-        <v>0.36499999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="D10" s="29">
         <f>SUM(D5:D9)</f>
-        <v>3.65</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -5671,7 +5701,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>187</v>
       </c>
@@ -5803,19 +5833,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="30">
         <v>46321</v>
       </c>
       <c r="B6" s="23">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>204</v>
       </c>
       <c r="D6" s="10">
         <f>SUM($B$4:B6)</f>
-        <v>22</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -5824,7 +5854,7 @@
       </c>
       <c r="B7" s="24">
         <f>SUM(B4:B6)</f>
-        <v>22</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>